<commit_message>
Fase 1: aplicar el contrato por ambiente con DDL no destructivo
- Contrato: el servidor databricks_dev se reemplaza por un servidor por
  ambiente (desa, prod) con la convención <ambiente>_<capa>.<subdominio>.
- Nuevo módulo databricks/contratos.py, reutilizable por capa: resuelve la
  tabla del ambiente, crea la tabla si no existe y solo aplica columnas
  opcionales nuevas (ALTER ADD COLUMNS); cualquier otra diferencia detiene
  el proceso. Gate, publicación por nombre de columna y validación.
- Notebook: widgets ambiente/escenario. Un gate fallido ya no vacía la
  tabla (antes el CREATE OR REPLACE corría antes del gate).
- Serverless: se fija pandas>=2.2,<3, que exige el motor de validación.

Probado en Databricks Free Edition serverless: ok (39/39), errores (8
fallidos, la tabla conserva sus filas), columna opcional nueva (ALTER,
41/41) y columna sobrante (se detiene sin tocar la tabla).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/alcance/landing_ded/ded_tarifario_prestacion.xlsx
+++ b/alcance/landing_ded/ded_tarifario_prestacion.xlsx
@@ -1424,10 +1424,14 @@
       </c>
       <c r="E4" s="35" t="inlineStr">
         <is>
-          <t>databricks_dev</t>
-        </is>
-      </c>
-      <c r="F4" s="35" t="n"/>
+          <t>desa</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
@@ -1494,10 +1498,14 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="F5" s="35" t="n"/>
+          <t>desa</t>
+        </is>
+      </c>
+      <c r="F5" s="35" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
@@ -1564,10 +1572,14 @@
       </c>
       <c r="E6" s="35" t="inlineStr">
         <is>
-          <t>Ambiente de pruebas en Databricks (Unity Catalog).</t>
-        </is>
-      </c>
-      <c r="F6" s="35" t="n"/>
+          <t>Ambiente de desarrollo en Databricks (Unity Catalog).</t>
+        </is>
+      </c>
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>Ambiente productivo en Databricks (Unity Catalog).</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
@@ -1691,7 +1703,11 @@
           <t>databricks</t>
         </is>
       </c>
-      <c r="F8" s="35" t="n"/>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>databricks</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -1920,10 +1936,14 @@
       <c r="D12" s="35" t="n"/>
       <c r="E12" s="35" t="inlineStr">
         <is>
-          <t>workspace</t>
-        </is>
-      </c>
-      <c r="F12" s="35" t="n"/>
+          <t>desa_landing</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>prod_landing</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
@@ -2864,10 +2884,14 @@
       <c r="D28" s="35" t="n"/>
       <c r="E28" s="35" t="inlineStr">
         <is>
-          <t>landing_ded</t>
-        </is>
-      </c>
-      <c r="F28" s="35" t="n"/>
+          <t>tarifarios</t>
+        </is>
+      </c>
+      <c r="F28" s="35" t="inlineStr">
+        <is>
+          <t>tarifarios</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
@@ -3278,10 +3302,14 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>databricks_dev</t>
-        </is>
-      </c>
-      <c r="F35" s="35" t="n"/>
+          <t>desa</t>
+        </is>
+      </c>
+      <c r="F35" s="35" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>

</xml_diff>